<commit_message>
feat: Centro de Comando Personal v2.0
Rediseno completo como plataforma ejecutiva corporativa:
- 7 modulos: Centro de Comando, Diagnostico de Riesgo, Bandeja Operacional,
  Seguimiento de Terceros, Reuniones, Productividad, Consumo de Tiempo
- Nueva arquitectura Excel: TAREAS (17 col) + TERCEROS + REUNIONES + REFERENCIA
- Diseno dark premium identico a dashboard Control de Aridos
- Matriz de riesgo Urgencia x Impacto con burbujas ECharts
- Estado general automatico: CONTROLADO / BAJO PRESION / CRITICO
- 39 tareas migradas con campos extendidos (IMPACTO, URGENCIA, ESFUERZO_HRS, TIPO, CATEGORIA, TERCERO)
- 6 terceros y 4 reuniones pre-cargadas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -8,7 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCIA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REUNIONES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCIA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +35,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="0038BDF8"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -60,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D1830"/>
+        <fgColor rgb="000A1220"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A1220"/>
+        <fgColor rgb="000D1830"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,31 +97,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,22 +505,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
@@ -513,46 +540,81 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TIPO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>AREA</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PRIORIDAD</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>FECHA_INICIO</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>IMPACTO</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>URGENCIA</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ESFUERZO_HRS</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>TERCERO</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA_CREACION</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>FECHA_COMPROMISO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FECHA_CIERRE</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -561,70 +623,122 @@
           <t>REVISIÓN plan de abastecimiento CL038</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Planificación</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M2" s="4" t="inlineStr"/>
+      <c r="N2" s="6" t="n">
+        <v>46180</v>
+      </c>
+      <c r="O2" s="6" t="n">
         <v>46192</v>
       </c>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="P2" s="5" t="n"/>
+      <c r="Q2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>SEGUIMIENTO correo clínica MEDs (carpeta rendición Isapre)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Completada</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="7" t="n">
+      <c r="J3" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Clínica MEDs</t>
+        </is>
+      </c>
+      <c r="N3" s="11" t="n">
+        <v>46179</v>
+      </c>
+      <c r="O3" s="11" t="n">
         <v>46186</v>
       </c>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+      <c r="P3" s="11" t="n">
+        <v>46186</v>
+      </c>
+      <c r="Q3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -633,286 +747,478 @@
           <t>LLEVAR formulario seguro (boletas terapía)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O4" s="6" t="n">
         <v>46189</v>
       </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>SEGUIMIENTO IConstruye (reportabilidad gastado a la fecha)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>ICONSTRUYE</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="7" t="n">
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>IConstruye</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>46181</v>
+      </c>
+      <c r="O5" s="11" t="n">
         <v>46188</v>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
+      <c r="P5" s="10" t="n"/>
+      <c r="Q5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>APROBAR contratos</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Contratos</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O6" s="6" t="n">
         <v>46187</v>
       </c>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Aprobar regularización equipos robados</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="7" t="n">
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="9" t="inlineStr"/>
+      <c r="N7" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O7" s="11" t="n">
         <v>46189</v>
       </c>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
+      <c r="P7" s="10" t="n"/>
+      <c r="Q7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>VISITAR a mi tío</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O8" s="6" t="n">
         <v>46187</v>
       </c>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>PASAR aspiradora</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="7" t="n">
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M9" s="9" t="inlineStr"/>
+      <c r="N9" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O9" s="11" t="n">
         <v>46187</v>
       </c>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+      <c r="P9" s="10" t="n"/>
+      <c r="Q9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>HACER baño 1</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O10" s="6" t="n">
         <v>46187</v>
       </c>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>ENVIAR correo presentación directorio (diferido)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>DIRECTORIO</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="7" t="n">
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Directorio</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O11" s="11" t="n">
         <v>46187</v>
       </c>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
+      <c r="P11" s="10" t="n"/>
+      <c r="Q11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -921,142 +1227,246 @@
           <t>SOLICITAR a GB respaldos de acta de sesión de Directorios</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>DIRECTORIO</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="4" t="n">
+      <c r="J12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O12" s="6" t="n">
         <v>46190</v>
       </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="n">
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>ACTUALIZAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Planificación</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="7" t="n">
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="9" t="inlineStr"/>
+      <c r="N13" s="11" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O13" s="11" t="n">
         <v>46187</v>
       </c>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
+      <c r="P13" s="10" t="n"/>
+      <c r="Q13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>RESERVA hora con Javi Franco</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>PERSONAL</t>
-        </is>
-      </c>
+      <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="4" t="n">
+      <c r="J14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Javi Franco</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O14" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>GESTIONAR firma MPD</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="7" t="n">
+      <c r="J15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>MPD</t>
+        </is>
+      </c>
+      <c r="N15" s="11" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O15" s="11" t="n">
         <v>46189</v>
       </c>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+      <c r="P15" s="10" t="n"/>
+      <c r="Q15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1065,70 +1475,120 @@
           <t>GESTIONAR firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Contratos</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="4" t="n">
+      <c r="J16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Salfa</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O16" s="6" t="n">
         <v>46189</v>
       </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>ENVIAR comunicado por día de vacaciones</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="7" t="n">
+      <c r="J17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M17" s="9" t="inlineStr"/>
+      <c r="N17" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O17" s="11" t="n">
         <v>46189</v>
       </c>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+      <c r="P17" s="10" t="n"/>
+      <c r="Q17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -1137,430 +1597,710 @@
           <t>PRESENTAR Dashboard Control de áridos</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O18" s="6" t="n">
         <v>46189</v>
       </c>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="P18" s="5" t="n"/>
+      <c r="Q18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>LAVAR ropa</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="7" t="n">
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M19" s="9" t="inlineStr"/>
+      <c r="N19" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O19" s="11" t="n">
         <v>46186</v>
       </c>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
+      <c r="P19" s="10" t="n"/>
+      <c r="Q19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>LAVAR losa</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="4" t="n">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O20" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 3/5</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="7" t="n">
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="9" t="inlineStr"/>
+      <c r="N21" s="11" t="n">
+        <v>46181</v>
+      </c>
+      <c r="O21" s="11" t="n">
         <v>46187</v>
       </c>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
+      <c r="P21" s="10" t="n"/>
+      <c r="Q21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 4/5</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="4" t="n">
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" s="6" t="n">
+        <v>46181</v>
+      </c>
+      <c r="O22" s="6" t="n">
         <v>46188</v>
       </c>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="5" t="n">
+      <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 5/5</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="7" t="n">
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="9" t="inlineStr"/>
+      <c r="N23" s="11" t="n">
+        <v>46181</v>
+      </c>
+      <c r="O23" s="11" t="n">
         <v>46189</v>
       </c>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
+      <c r="P23" s="10" t="n"/>
+      <c r="Q23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>BARRER hojas</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="4" t="n">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O24" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="5" t="n">
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>PREPARAR almuerzo</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="7" t="n">
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M25" s="9" t="inlineStr"/>
+      <c r="N25" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O25" s="11" t="n">
         <v>46186</v>
       </c>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
+      <c r="P25" s="10" t="n"/>
+      <c r="Q25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 2/5</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="4" t="n">
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" s="4" t="inlineStr"/>
+      <c r="N26" s="6" t="n">
+        <v>46181</v>
+      </c>
+      <c r="O26" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="5" t="n">
+      <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>LLAMAR a Claudio S.</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr"/>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="7" t="n">
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>Claudio S.</t>
+        </is>
+      </c>
+      <c r="N27" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O27" s="11" t="n">
         <v>46186</v>
       </c>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
+      <c r="P27" s="10" t="n"/>
+      <c r="Q27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>ASISTIR cumpleaños Felipe M.</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="4" t="n">
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O28" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="5" t="n">
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>ASISTIR cumpleaños Esteban</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr"/>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="7" t="n">
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="9" t="inlineStr"/>
+      <c r="N29" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O29" s="11" t="n">
         <v>46186</v>
       </c>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30" ht="18" customHeight="1">
+      <c r="P29" s="10" t="n"/>
+      <c r="Q29" s="9" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
@@ -1569,70 +2309,120 @@
           <t>ENVIAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Planificación</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="4" t="n">
+      <c r="J30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O30" s="6" t="n">
         <v>46189</v>
       </c>
-      <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="5" t="n">
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>PRESENTAR carpetas 2 ciclos fertilización en isapre</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr"/>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="7" t="n">
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>Isapre</t>
+        </is>
+      </c>
+      <c r="N31" s="11" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O31" s="11" t="n">
         <v>46193</v>
       </c>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
+      <c r="P31" s="10" t="n"/>
+      <c r="Q31" s="9" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
@@ -1641,70 +2431,120 @@
           <t>REVISIÓN funcionamiento KIT en IConstruye</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>ICONSTRUYE</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="4" t="n">
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>IConstruye</t>
+        </is>
+      </c>
+      <c r="N32" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O32" s="6" t="n">
         <v>46191</v>
       </c>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="5" t="n">
+      <c r="P32" s="5" t="n"/>
+      <c r="Q32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>ACTUALIZAR modelo Claude (validar datos)</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr"/>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="7" t="n">
+      <c r="J33" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" s="9" t="inlineStr"/>
+      <c r="N33" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O33" s="11" t="n">
         <v>46187</v>
       </c>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="inlineStr"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
+      <c r="P33" s="10" t="n"/>
+      <c r="Q33" s="9" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
@@ -1713,142 +2553,238 @@
           <t>COORDINAR hora psiquiatra (Consultar con la Lore)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="4" t="n">
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Consultorio</t>
+        </is>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O34" s="6" t="n">
         <v>46186</v>
       </c>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="5" t="n">
+      <c r="P34" s="5" t="n"/>
+      <c r="Q34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>COMPRAR nuevo anillo matrimonial</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr"/>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="7" t="n">
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="9" t="inlineStr"/>
+      <c r="N35" s="11" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O35" s="11" t="n">
         <v>46193</v>
       </c>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
+      <c r="P35" s="10" t="n"/>
+      <c r="Q35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>ENVIAR a reparar bicicleta</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="4" t="n">
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="O36" s="6" t="n">
         <v>46193</v>
       </c>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="5" t="n">
+      <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>ENTRENAR trote: Rodaje 5K (Matutino)</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr"/>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="7" t="n">
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" s="9" t="inlineStr"/>
+      <c r="N37" s="11" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O37" s="11" t="n">
         <v>46188</v>
       </c>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
+      <c r="P37" s="10" t="n"/>
+      <c r="Q37" s="9" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
@@ -1857,68 +2793,114 @@
           <t>ARMAR propuesta para salida fin de mes</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="4" t="n">
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="O38" s="6" t="n">
         <v>46187</v>
       </c>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="5" t="n">
+      <c r="P38" s="5" t="n"/>
+      <c r="Q38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Revisar propuestas PUC RSC</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr"/>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="inlineStr"/>
-    </row>
-    <row r="40" ht="18" customHeight="1">
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" s="9" t="inlineStr"/>
+      <c r="N39" s="11" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O39" s="10" t="n"/>
+      <c r="P39" s="10" t="n"/>
+      <c r="Q39" s="9" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
@@ -1927,30 +2909,53 @@
           <t>Consolidar ensayos Mov. Tierra CL027</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>CL027</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Planificación</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="O40" s="5" t="n"/>
+      <c r="P40" s="5" t="n"/>
+      <c r="Q40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1963,147 +2968,933 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NOMBRE</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIZACION</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ROL</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TEMA_PENDIENTE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA_INICIO_SEG</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA_ULTIMO_SEG</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ESTADO</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PRIORIDAD</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>IConstruye</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Digital</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Proveedor de Servicio</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Funcionamiento KIT y reporte reportabilidad</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>46182</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Abrir ticket si no responden en 48h</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Gerencia Buenos Aires</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Gerencia Corporativa</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Respaldos actas de sesión Directorio</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46183</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>Recordar para reunión directorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>MPD</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Mandante Proyecto</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Mandante</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Firma contrato pendiente</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>46182</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Bloquea inicio de faena</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Salfa</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Salfa Contratistas</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Contratista</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Firma Contrato Salfa-Londres</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46182</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Coordinar con legal si hay demora</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Isapre</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Institución de Salud</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Institución Salud</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Presentación carpetas 2 ciclos fertilización</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>46179</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>46179</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Plazo vence 20 junio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Clínica MEDs</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Clínica Médica</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Prestador Salud</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Correo rendición Isapre</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46179</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>46186</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Correo recibido</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>TITULO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TIPO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PARTICIPANTES</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ESTADO</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>COMPROMISO</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>RESPONSABLE_COMP</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA_COMP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ESTADO_COMP</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Reunión Directorio — Estado de Obras</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>46193</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Directorio</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Gerencia, Directores, ITO</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Preparar presentación estado obras; Enviar correo previo con agenda</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="n">
+        <v>46191</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Presentar avance CL038 y CL027</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Coordinación Avance CL038</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>46190</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Obra</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>ITO, Administrador de Obra, Subcontratistas</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Enviar informe de avance; Actualizar formato hormigones</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Revisar plan de abastecimiento áridos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Revisión Contratos — Salfa / MPD</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>46189</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Contratos</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Gerencia, Asesor Legal, Representante Salfa</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Gestionar firma MPD; Gestionar firma Salfa; Enviar copia a legal</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>46188</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar asistencia de ambas partes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Seguimiento IConstruye — Funcionalidades</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>46191</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Soporte IConstruye, Planificación</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Resolver funcionamiento KIT; Revisar reportabilidad gastado</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>46191</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>Preparar pantallazos con el error</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PRIORIDAD</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>AREA</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TIPO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>IMPACTO</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>URGENCIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Crítica</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Planificación</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>1 - Mínimo</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>1 - Sin urgencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>CL027</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Contratos</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>2 - Bajo</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>2 - Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>ICONSTRUYE</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Esperando Terceros</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>3 - Medio</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>3 - Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Completada</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Reunión</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>4 - Alto</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>4 - Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Cancelada</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>IA y Automatización</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>5 - Crítico</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>5 - Inmediata</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>DIRECTORIO</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Reuniones</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Personal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 06:16)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REUNIONES" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCIA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="REUNIONES" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +19,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,47 +30,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0038BDF8"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00CBD5E1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="0094A3B8"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000D1526"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000A1220"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000D1830"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -79,67 +47,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="001E293B"/>
-      </left>
-      <right style="thin">
-        <color rgb="001E293B"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E293B"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001E293B"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,2455 +421,2436 @@
   </sheetPr>
   <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>TAREA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>PROYECTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>AREA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>CATEGORIA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>PRIORIDAD</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>IMPACTO</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>URGENCIA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ESFUERZO_HRS</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>TERCERO</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>FECHA_CREACION</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>FECHA_COMPROMISO</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>FECHA_CIERRE</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>REVISIÓN plan de abastecimiento CL038</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Planificación</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" t="n">
         <v>4</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" t="n">
         <v>1.5</v>
       </c>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="6" t="n">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="O2" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="P2" s="5" t="n"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="7" t="n">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>SEGUIMIENTO correo clínica MEDs (carpeta rendición Isapre)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Completada</t>
         </is>
       </c>
-      <c r="J3" s="7" t="n">
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="7" t="n">
+      <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" s="7" t="n">
+      <c r="L3" t="n">
         <v>0.5</v>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Clínica MEDs</t>
         </is>
       </c>
-      <c r="N3" s="11" t="n">
+      <c r="N3" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="O3" s="11" t="n">
+      <c r="O3" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P3" s="11" t="n">
+      <c r="P3" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="Q3" s="9" t="inlineStr"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="Q3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>LLEVAR formulario seguro (boletas terapía)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
         <v>3</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" t="n">
         <v>4</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" t="n">
         <v>0.5</v>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="6" t="n">
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="O4" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="7" t="n">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>SEGUIMIENTO IConstruye (reportabilidad gastado a la fecha)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>ICONSTRUYE</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Reportes</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="n">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
         <v>3</v>
       </c>
-      <c r="K5" s="7" t="n">
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="7" t="n">
+      <c r="L5" t="n">
         <v>1</v>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="N5" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O5" s="11" t="n">
+      <c r="O5" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>APROBAR contratos</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Contratos</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="6" t="n">
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="O6" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Aprobar regularización equipos robados</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="n">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
         <v>3</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K7" t="n">
         <v>4</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="9" t="inlineStr"/>
-      <c r="N7" s="11" t="n">
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O7" s="11" t="n">
+      <c r="O7" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P7" s="10" t="n"/>
-      <c r="Q7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="n">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>VISITAR a mi tío</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="n">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" t="n">
         <v>5</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="L8" t="n">
         <v>2</v>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="6" t="n">
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O8" s="6" t="n">
+      <c r="O8" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="7" t="n">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>PASAR aspiradora</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="n">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="K9" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="7" t="n">
+      <c r="L9" t="n">
         <v>0.5</v>
       </c>
-      <c r="M9" s="9" t="inlineStr"/>
-      <c r="N9" s="11" t="n">
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O9" s="11" t="n">
+      <c r="O9" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P9" s="10" t="n"/>
-      <c r="Q9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="n">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>HACER baño 1</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="n">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" t="n">
         <v>5</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="L10" t="n">
         <v>0.5</v>
       </c>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="6" t="n">
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O10" s="6" t="n">
+      <c r="O10" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P10" s="5" t="n"/>
-      <c r="Q10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>ENVIAR correo presentación directorio (diferido)</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>DIRECTORIO</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="n">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
         <v>4</v>
       </c>
-      <c r="K11" s="7" t="n">
+      <c r="K11" t="n">
         <v>5</v>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="L11" t="n">
         <v>0.5</v>
       </c>
-      <c r="M11" s="9" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Directorio</t>
         </is>
       </c>
-      <c r="N11" s="11" t="n">
+      <c r="N11" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O11" s="11" t="n">
+      <c r="O11" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P11" s="10" t="n"/>
-      <c r="Q11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>SOLICITAR a GB respaldos de acta de sesión de Directorios</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>DIRECTORIO</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" t="n">
         <v>4</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" t="n">
         <v>4</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="L12" t="n">
         <v>0.5</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="N12" s="6" t="n">
+      <c r="N12" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O12" s="6" t="n">
+      <c r="O12" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="P12" s="5" t="n"/>
-      <c r="Q12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="7" t="n">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>ACTUALIZAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Planificación</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="n">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="7" t="n">
+      <c r="K13" t="n">
         <v>5</v>
       </c>
-      <c r="L13" s="7" t="n">
+      <c r="L13" t="n">
         <v>2</v>
       </c>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="11" t="n">
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O13" s="11" t="n">
+      <c r="O13" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P13" s="10" t="n"/>
-      <c r="Q13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="n">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>RESERVA hora con Javi Franco</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" t="n">
         <v>5</v>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="L14" t="n">
         <v>0.5</v>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Javi Franco</t>
         </is>
       </c>
-      <c r="N14" s="6" t="n">
+      <c r="N14" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O14" s="6" t="n">
+      <c r="O14" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P14" s="5" t="n"/>
-      <c r="Q14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="7" t="n">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>GESTIONAR firma MPD</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" t="n">
         <v>4</v>
       </c>
-      <c r="K15" s="7" t="n">
+      <c r="K15" t="n">
         <v>4</v>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="L15" t="n">
         <v>1.5</v>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>MPD</t>
         </is>
       </c>
-      <c r="N15" s="11" t="n">
+      <c r="N15" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O15" s="11" t="n">
+      <c r="O15" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P15" s="10" t="n"/>
-      <c r="Q15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="n">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>GESTIONAR firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Contratos</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J16" t="n">
         <v>5</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" t="n">
         <v>4</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="L16" t="n">
         <v>1.5</v>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Salfa</t>
         </is>
       </c>
-      <c r="N16" s="6" t="n">
+      <c r="N16" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O16" s="6" t="n">
+      <c r="O16" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P16" s="5" t="n"/>
-      <c r="Q16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>ENVIAR comunicado por día de vacaciones</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J17" s="7" t="n">
+      <c r="J17" t="n">
         <v>4</v>
       </c>
-      <c r="K17" s="7" t="n">
+      <c r="K17" t="n">
         <v>4</v>
       </c>
-      <c r="L17" s="7" t="n">
+      <c r="L17" t="n">
         <v>0.5</v>
       </c>
-      <c r="M17" s="9" t="inlineStr"/>
-      <c r="N17" s="11" t="n">
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O17" s="11" t="n">
+      <c r="O17" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P17" s="10" t="n"/>
-      <c r="Q17" s="9" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="n">
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>PRESENTAR Dashboard Control de áridos</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
         <v>4</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K18" t="n">
         <v>4</v>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="L18" t="n">
         <v>2</v>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="6" t="n">
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O18" s="6" t="n">
+      <c r="O18" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P18" s="5" t="n"/>
-      <c r="Q18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>LAVAR ropa</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="n">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
         <v>1</v>
       </c>
-      <c r="K19" s="7" t="n">
+      <c r="K19" t="n">
         <v>5</v>
       </c>
-      <c r="L19" s="7" t="n">
+      <c r="L19" t="n">
         <v>0.5</v>
       </c>
-      <c r="M19" s="9" t="inlineStr"/>
-      <c r="N19" s="11" t="n">
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O19" s="11" t="n">
+      <c r="O19" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P19" s="10" t="n"/>
-      <c r="Q19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="n">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>LAVAR losa</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="n">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="K20" t="n">
         <v>5</v>
       </c>
-      <c r="L20" s="2" t="n">
+      <c r="L20" t="n">
         <v>0.5</v>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="6" t="n">
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O20" s="6" t="n">
+      <c r="O20" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P20" s="5" t="n"/>
-      <c r="Q20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 3/5</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr"/>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="n">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
         <v>3</v>
       </c>
-      <c r="K21" s="7" t="n">
+      <c r="K21" t="n">
         <v>5</v>
       </c>
-      <c r="L21" s="7" t="n">
+      <c r="L21" t="n">
         <v>2</v>
       </c>
-      <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="11" t="n">
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O21" s="11" t="n">
+      <c r="O21" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P21" s="10" t="n"/>
-      <c r="Q21" s="9" t="inlineStr"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="2" t="n">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 4/5</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="n">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
         <v>3</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" t="n">
         <v>5</v>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="L22" t="n">
         <v>2</v>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="6" t="n">
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O22" s="6" t="n">
+      <c r="O22" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P22" s="5" t="n"/>
-      <c r="Q22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 5/5</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr"/>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="n">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="K23" t="n">
         <v>4</v>
       </c>
-      <c r="L23" s="7" t="n">
+      <c r="L23" t="n">
         <v>2</v>
       </c>
-      <c r="M23" s="9" t="inlineStr"/>
-      <c r="N23" s="11" t="n">
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O23" s="11" t="n">
+      <c r="O23" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P23" s="10" t="n"/>
-      <c r="Q23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="2" t="n">
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>BARRER hojas</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="n">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" t="n">
         <v>5</v>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="L24" t="n">
         <v>0.5</v>
       </c>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="6" t="n">
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O24" s="6" t="n">
+      <c r="O24" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P24" s="5" t="n"/>
-      <c r="Q24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="7" t="n">
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>PREPARAR almuerzo</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="n">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="7" t="n">
+      <c r="K25" t="n">
         <v>5</v>
       </c>
-      <c r="L25" s="7" t="n">
+      <c r="L25" t="n">
         <v>0.5</v>
       </c>
-      <c r="M25" s="9" t="inlineStr"/>
-      <c r="N25" s="11" t="n">
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O25" s="11" t="n">
+      <c r="O25" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P25" s="10" t="n"/>
-      <c r="Q25" s="9" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="2" t="n">
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>CAPACITACIÓN Claude Code 2/5</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="n">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
         <v>3</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="K26" t="n">
         <v>5</v>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="L26" t="n">
         <v>2</v>
       </c>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="6" t="n">
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O26" s="6" t="n">
+      <c r="O26" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P26" s="5" t="n"/>
-      <c r="Q26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="n">
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>LLAMAR a Claudio S.</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="n">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
         <v>3</v>
       </c>
-      <c r="K27" s="7" t="n">
+      <c r="K27" t="n">
         <v>5</v>
       </c>
-      <c r="L27" s="7" t="n">
+      <c r="L27" t="n">
         <v>0.5</v>
       </c>
-      <c r="M27" s="9" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>Claudio S.</t>
         </is>
       </c>
-      <c r="N27" s="11" t="n">
+      <c r="N27" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O27" s="11" t="n">
+      <c r="O27" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P27" s="10" t="n"/>
-      <c r="Q27" s="9" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="n">
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>ASISTIR cumpleaños Felipe M.</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="n">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
         <v>2</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="K28" t="n">
         <v>5</v>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="L28" t="n">
         <v>2</v>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="6" t="n">
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O28" s="6" t="n">
+      <c r="O28" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P28" s="5" t="n"/>
-      <c r="Q28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="7" t="n">
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>ASISTIR cumpleaños Esteban</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr"/>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J29" s="7" t="n">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
         <v>2</v>
       </c>
-      <c r="K29" s="7" t="n">
+      <c r="K29" t="n">
         <v>5</v>
       </c>
-      <c r="L29" s="7" t="n">
+      <c r="L29" t="n">
         <v>2</v>
       </c>
-      <c r="M29" s="9" t="inlineStr"/>
-      <c r="N29" s="11" t="n">
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O29" s="11" t="n">
+      <c r="O29" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P29" s="10" t="n"/>
-      <c r="Q29" s="9" t="inlineStr"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="2" t="n">
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>ENVIAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>CL038</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Planificación</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n">
+      <c r="J30" t="n">
         <v>3</v>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="K30" t="n">
         <v>4</v>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="L30" t="n">
         <v>0.5</v>
       </c>
-      <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="6" t="n">
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O30" s="6" t="n">
+      <c r="O30" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P30" s="5" t="n"/>
-      <c r="Q30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="7" t="n">
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>PRESENTAR carpetas 2 ciclos fertilización en isapre</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr"/>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="n">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
         <v>4</v>
       </c>
-      <c r="K31" s="7" t="n">
+      <c r="K31" t="n">
         <v>3</v>
       </c>
-      <c r="L31" s="7" t="n">
+      <c r="L31" t="n">
         <v>2</v>
       </c>
-      <c r="M31" s="9" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Isapre</t>
         </is>
       </c>
-      <c r="N31" s="11" t="n">
+      <c r="N31" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O31" s="11" t="n">
+      <c r="O31" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="P31" s="10" t="n"/>
-      <c r="Q31" s="9" t="inlineStr"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="2" t="n">
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>REVISIÓN funcionamiento KIT en IConstruye</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>ICONSTRUYE</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Reportes</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="n">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
         <v>3</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" t="n">
         <v>3</v>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="L32" t="n">
         <v>1.5</v>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N32" s="6" t="n">
+      <c r="N32" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O32" s="6" t="n">
+      <c r="O32" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="P32" s="5" t="n"/>
-      <c r="Q32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="7" t="n">
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>ACTUALIZAR modelo Claude (validar datos)</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr"/>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>AGENTE_IA</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>IA y Automatización</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="J33" s="7" t="n">
+      <c r="J33" t="n">
         <v>3</v>
       </c>
-      <c r="K33" s="7" t="n">
+      <c r="K33" t="n">
         <v>5</v>
       </c>
-      <c r="L33" s="7" t="n">
+      <c r="L33" t="n">
         <v>2</v>
       </c>
-      <c r="M33" s="9" t="inlineStr"/>
-      <c r="N33" s="11" t="n">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O33" s="11" t="n">
+      <c r="O33" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P33" s="10" t="n"/>
-      <c r="Q33" s="9" t="inlineStr"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="2" t="n">
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>COORDINAR hora psiquiatra (Consultar con la Lore)</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>SALUD</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="n">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
         <v>3</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" t="n">
         <v>5</v>
       </c>
-      <c r="L34" s="2" t="n">
+      <c r="L34" t="n">
         <v>0.5</v>
       </c>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>Consultorio</t>
         </is>
       </c>
-      <c r="N34" s="6" t="n">
+      <c r="N34" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O34" s="6" t="n">
+      <c r="O34" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P34" s="5" t="n"/>
-      <c r="Q34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="7" t="n">
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>COMPRAR nuevo anillo matrimonial</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr"/>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="n">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
         <v>2</v>
       </c>
-      <c r="K35" s="7" t="n">
+      <c r="K35" t="n">
         <v>3</v>
       </c>
-      <c r="L35" s="7" t="n">
+      <c r="L35" t="n">
         <v>1</v>
       </c>
-      <c r="M35" s="9" t="inlineStr"/>
-      <c r="N35" s="11" t="n">
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O35" s="11" t="n">
+      <c r="O35" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="P35" s="10" t="n"/>
-      <c r="Q35" s="9" t="inlineStr"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="2" t="n">
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>ENVIAR a reparar bicicleta</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="n">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
         <v>2</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="K36" t="n">
         <v>3</v>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="L36" t="n">
         <v>0.5</v>
       </c>
-      <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="6" t="n">
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O36" s="6" t="n">
+      <c r="O36" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="P36" s="5" t="n"/>
-      <c r="Q36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="7" t="n">
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>ENTRENAR trote: Rodaje 5K (Matutino)</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr"/>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J37" s="7" t="n">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
         <v>3</v>
       </c>
-      <c r="K37" s="7" t="n">
+      <c r="K37" t="n">
         <v>5</v>
       </c>
-      <c r="L37" s="7" t="n">
+      <c r="L37" t="n">
         <v>1</v>
       </c>
-      <c r="M37" s="9" t="inlineStr"/>
-      <c r="N37" s="11" t="n">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O37" s="11" t="n">
+      <c r="O37" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P37" s="10" t="n"/>
-      <c r="Q37" s="9" t="inlineStr"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="2" t="n">
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>ARMAR propuesta para salida fin de mes</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>PERSONAL</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="n">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
         <v>3</v>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="K38" t="n">
         <v>5</v>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="L38" t="n">
         <v>1.5</v>
       </c>
-      <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="6" t="n">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O38" s="6" t="n">
+      <c r="O38" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P38" s="5" t="n"/>
-      <c r="Q38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="7" t="n">
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Revisar propuestas PUC RSC</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr"/>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>CORPORATIVO</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Gestión Corporativa</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="n">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
         <v>3</v>
       </c>
-      <c r="K39" s="7" t="n">
+      <c r="K39" t="n">
         <v>1</v>
       </c>
-      <c r="L39" s="7" t="n">
+      <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="M39" s="9" t="inlineStr"/>
-      <c r="N39" s="11" t="n">
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O39" s="10" t="n"/>
-      <c r="P39" s="10" t="n"/>
-      <c r="Q39" s="9" t="inlineStr"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="2" t="n">
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Consolidar ensayos Mov. Tierra CL027</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>CL027</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Trabajo</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Planificación</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="n">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
         <v>3</v>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="K40" t="n">
         <v>1</v>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="L40" t="n">
         <v>2</v>
       </c>
-      <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="6" t="n">
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O40" s="5" t="n"/>
-      <c r="P40" s="5" t="n"/>
-      <c r="Q40" s="4" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2970,342 +2865,330 @@
   </sheetPr>
   <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ORGANIZACION</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ROL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>TEMA_PENDIENTE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>FECHA_INICIO_SEG</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>FECHA_ULTIMO_SEG</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>PRIORIDAD</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Plataforma Digital</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Proveedor de Servicio</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Funcionamiento KIT y reporte reportabilidad</t>
         </is>
       </c>
-      <c r="F2" s="12" t="n">
+      <c r="F2" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G2" s="12" t="n">
+      <c r="G2" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Abrir ticket si no responden en 48h</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="7" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Gerencia Buenos Aires</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Gerencia Corporativa</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Respaldos actas de sesión Directorio</t>
         </is>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="G3" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Recordar para reunión directorio</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>MPD</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mandante Proyecto</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Mandante</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Firma contrato pendiente</t>
         </is>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Bloquea inicio de faena</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="7" t="n">
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Salfa</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Salfa Contratistas</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Contratista</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Coordinar con legal si hay demora</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="6">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Isapre</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Institución de Salud</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Institución Salud</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Presentación carpetas 2 ciclos fertilización</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Plazo vence 20 junio</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="7" t="n">
+    <row r="7">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Clínica MEDs</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Clínica Médica</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Prestador Salud</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Correo rendición Isapre</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Resuelto</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Correo recibido</t>
         </is>
@@ -3324,577 +3207,265 @@
   </sheetPr>
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>TITULO</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>PARTICIPANTES</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>COMPROMISO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>RESPONSABLE_COMP</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>FECHA_COMP</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ESTADO_COMP</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Reunión Directorio — Estado de Obras</t>
         </is>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Directorio</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Gerencia, Directores, ITO</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Preparar presentación estado obras; Enviar correo previo con agenda</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Juan</t>
         </is>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="I2" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Presentar avance CL038 y CL027</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Coordinación Avance CL038</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Obra</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>ITO, Administrador de Obra, Subcontratistas</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Enviar informe de avance; Actualizar formato hormigones</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Juan</t>
         </is>
       </c>
-      <c r="I3" s="13" t="n">
+      <c r="I3" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Revisar plan de abastecimiento áridos</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Revisión Contratos — Salfa / MPD</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Contratos</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Gerencia, Asesor Legal, Representante Salfa</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Gestionar firma MPD; Gestionar firma Salfa; Enviar copia a legal</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Juan</t>
         </is>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Confirmar asistencia de ambas partes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="7" t="n">
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Seguimiento IConstruye — Funcionalidades</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Tecnología</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Soporte IConstruye, Planificación</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>Resolver funcionamiento KIT; Revisar reportabilidad gastado</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Juan</t>
         </is>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Preparar pantallazos con el error</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PROYECTO</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>PRIORIDAD</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>ESTADO</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>AREA</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>TIPO</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CATEGORIA</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IMPACTO</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>URGENCIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>CL038</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Crítica</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>Trabajo</t>
-        </is>
-      </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>Planificación</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>1 - Mínimo</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>1 - Sin urgencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>CL027</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>En Proceso</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="E3" s="15" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="inlineStr">
-        <is>
-          <t>Contratos</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="inlineStr">
-        <is>
-          <t>2 - Bajo</t>
-        </is>
-      </c>
-      <c r="H3" s="15" t="inlineStr">
-        <is>
-          <t>2 - Baja</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>ICONSTRUYE</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Esperando Terceros</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Compromiso</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>3 - Medio</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>3 - Media</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>AGENTE_IA</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Completada</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>Reunión</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Reportes</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>4 - Alto</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>4 - Alta</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>CORPORATIVO</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Cancelada</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>IA y Automatización</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>5 - Crítico</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>5 - Inmediata</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>DIRECTORIO</t>
-        </is>
-      </c>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>Gestión Corporativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>SALUD</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>Reuniones</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>PERSONAL</t>
-        </is>
-      </c>
-      <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>Salud</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>Personal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 06:17)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J20" t="n">
@@ -1661,7 +1661,9 @@
       <c r="O20" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 16:53)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2486,7 +2486,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J34" t="n">
@@ -2509,7 +2509,9 @@
       <c r="O34" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 16:59)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2673,7 +2673,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2692,7 +2692,9 @@
       <c r="O37" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 17:34)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -752,7 +752,9 @@
       <c r="O5" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 18:06)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Completada</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -794,7 +794,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Completada</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="J6" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 18:33)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,6 +508,11 @@
           <t>NOTAS</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>COMENTARIOS</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -567,6 +572,7 @@
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -632,6 +638,7 @@
         <v>46186</v>
       </c>
       <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -691,6 +698,7 @@
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -756,6 +764,7 @@
         <v>46187</v>
       </c>
       <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -817,6 +826,7 @@
         <v>46187</v>
       </c>
       <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -876,6 +886,7 @@
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -935,6 +946,7 @@
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -994,6 +1006,7 @@
       </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1053,6 +1066,7 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1116,6 +1130,7 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1179,6 +1194,7 @@
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1238,6 +1254,7 @@
       </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1303,6 +1320,7 @@
         <v>46187</v>
       </c>
       <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1366,6 +1384,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1429,6 +1448,7 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1488,6 +1508,7 @@
       </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1547,6 +1568,7 @@
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1608,6 +1630,7 @@
         <v>46187</v>
       </c>
       <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1669,6 +1692,7 @@
         <v>46187</v>
       </c>
       <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1728,6 +1752,7 @@
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1787,6 +1812,7 @@
       </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1846,6 +1872,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1907,6 +1934,7 @@
         <v>46187</v>
       </c>
       <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1966,6 +1994,7 @@
       </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2025,6 +2054,7 @@
       </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2088,6 +2118,7 @@
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2147,6 +2178,7 @@
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2208,6 +2240,7 @@
         <v>46187</v>
       </c>
       <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2267,6 +2300,7 @@
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2330,6 +2364,7 @@
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2393,6 +2428,7 @@
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2452,6 +2488,7 @@
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2515,6 +2552,7 @@
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2574,6 +2612,7 @@
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2633,6 +2672,7 @@
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2692,6 +2732,7 @@
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2751,6 +2792,7 @@
       </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2808,6 +2850,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2865,6 +2908,7 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 18:47)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1293,7 +1293,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Completada</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1316,9 +1316,7 @@
       <c r="O14" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P14" s="1" t="n">
-        <v>46187</v>
-      </c>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 21:16)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1004,7 +1004,9 @@
       <c r="O9" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 21:25)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2909,6 +2909,66 @@
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PEDIR hora psiquiatra</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>3</v>
+      </c>
+      <c r="K41" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" s="1" t="n">
+        <v>46187</v>
+      </c>
+      <c r="O41" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 21:27)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2969,6 +2969,66 @@
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>COMPRAR parafina</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K42" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" s="1" t="n">
+        <v>46187</v>
+      </c>
+      <c r="O42" s="1" t="n">
+        <v>46187</v>
+      </c>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 22:29)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1973,7 +1973,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J25" t="n">
@@ -1992,7 +1992,9 @@
       <c r="O25" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (14/06 22:30)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2531,7 +2531,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J34" t="n">
@@ -2554,7 +2554,9 @@
       <c r="O34" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" s="1" t="n">
+        <v>46187</v>
+      </c>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 02:08)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1107,7 +1107,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1130,7 +1130,9 @@
       <c r="O11" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 02:12)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3039,6 +3039,56 @@
       </c>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ENVIAR correo a Julián por empresa seguridad Moreno</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O43" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 02:14)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3055,7 +3055,11 @@
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>Trabajo</t>
@@ -3076,9 +3080,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="J43" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" t="n">
+        <v>3</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" s="1" t="n">
         <v>46188</v>
@@ -3089,6 +3099,54 @@
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>REVISIÓN  con asesor de auto evaluación Sello PRO</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Reuniones</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 16:35)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -783,7 +783,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CORPORATIVO</t>
+          <t>CL034</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -820,7 +820,7 @@
         <v>46183</v>
       </c>
       <c r="O6" s="1" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="P6" s="1" t="n">
         <v>46187</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 16:37)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1064,7 +1064,7 @@
         <v>46185</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
@@ -2796,7 +2796,7 @@
         <v>46185</v>
       </c>
       <c r="O38" s="1" t="n">
-        <v>46188</v>
+        <v>46187</v>
       </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 16:39)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -1568,7 +1568,9 @@
       <c r="O18" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 16:40)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2721,7 +2721,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2740,7 +2740,9 @@
       <c r="O37" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 16:51)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3081,7 +3081,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J43" t="n">
@@ -3100,7 +3100,9 @@
       <c r="O43" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P43" t="inlineStr"/>
+      <c r="P43" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 18:41)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3165,6 +3165,56 @@
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ENVIAR pronostico polla mundialera 15-6-26</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O45" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 21:15)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -823,7 +823,7 @@
         <v>46188</v>
       </c>
       <c r="P6" s="1" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
@@ -3181,7 +3181,11 @@
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3202,9 +3206,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="J45" t="n">
+        <v>3</v>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1</v>
+      </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" s="1" t="n">
         <v>46188</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (15/06 21:42)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3225,6 +3225,56 @@
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>CORRER 7K</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O46" s="1" t="n">
+        <v>46194</v>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (16/06 00:45)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3203,7 +3203,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J45" t="n">
@@ -3222,7 +3222,9 @@
       <c r="O45" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P45" t="inlineStr"/>
+      <c r="P45" s="1" t="n">
+        <v>46189</v>
+      </c>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
     </row>
@@ -3241,7 +3243,11 @@
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3262,9 +3268,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="J46" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>3</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1</v>
+      </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" s="1" t="n">
         <v>46188</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (16/06 02:50)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2039,7 +2039,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -2058,7 +2058,9 @@
       <c r="O26" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" s="1" t="n">
+        <v>46189</v>
+      </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (17/06 19:32)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3289,6 +3289,60 @@
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ACTUALIZAR  Plan de Abastecimiento</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CL038</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="O47" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (18/06 13:38)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -694,7 +694,7 @@
         <v>46183</v>
       </c>
       <c r="O4" s="1" t="n">
-        <v>46189</v>
+        <v>46196</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
@@ -3330,9 +3330,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>3</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1</v>
+      </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" s="1" t="n">
         <v>46190</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (18/06 13:39)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -865,7 +865,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -884,7 +884,9 @@
       <c r="O7" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" s="1" t="n">
+        <v>46191</v>
+      </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (18/06 13:41)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3147,7 +3147,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J44" t="n">
@@ -3166,7 +3166,9 @@
       <c r="O44" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="P44" t="inlineStr"/>
+      <c r="P44" s="1" t="n">
+        <v>46191</v>
+      </c>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 00:26)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1491,7 +1491,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J17" t="n">
@@ -1510,7 +1510,9 @@
       <c r="O17" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 00:36)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:R48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3359,6 +3359,60 @@
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>APROBAR EEPP</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Of. Central</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O48" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 00:38)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R48"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3400,9 +3400,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>3</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" s="1" t="n">
         <v>46195</v>
@@ -3413,6 +3419,60 @@
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>APROBAR OC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>CL038</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O49" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 00:39)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3460,9 +3460,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="J49" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1</v>
+      </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" s="1" t="n">
         <v>46195</v>
@@ -3473,6 +3479,60 @@
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>APROBAR contratos</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Of. Central</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O50" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 00:40)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1876,7 +1876,7 @@
         <v>46181</v>
       </c>
       <c r="O23" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
@@ -3520,9 +3520,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="J50" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" t="n">
+        <v>3</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1</v>
+      </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" s="1" t="n">
         <v>46195</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:13)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3539,6 +3539,56 @@
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>VIAJAR a Olmue</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O51" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:14)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3555,7 +3555,11 @@
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3576,9 +3580,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="J51" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1</v>
+      </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" s="1" t="n">
         <v>46195</v>
@@ -3589,6 +3599,56 @@
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>LAVAR ropa</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O52" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:16)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3615,7 +3615,11 @@
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3636,9 +3640,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" s="1" t="n">
         <v>46195</v>
@@ -3649,6 +3659,56 @@
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ENTRENAMIENTO fuerza</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O53" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:17)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2126,7 +2126,7 @@
         <v>46185</v>
       </c>
       <c r="O27" s="1" t="n">
-        <v>46195</v>
+        <v>46199</v>
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
@@ -3675,7 +3675,11 @@
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3696,9 +3700,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1</v>
+      </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" s="1" t="n">
         <v>46195</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:18)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3719,6 +3719,56 @@
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>VISITAR escuela construcción PUC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O54" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:19)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3735,7 +3735,11 @@
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>Trabajo</t>
@@ -3748,7 +3752,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3756,9 +3760,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="J54" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" t="n">
+        <v>3</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1</v>
+      </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" s="1" t="n">
         <v>46195</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 01:57)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PEDIR hora psiquiatra</t>
+          <t>ASISTIR hora psiquiatra (14 hrs. Lo Barnechea)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -2984,7 +2984,7 @@
         <v>46187</v>
       </c>
       <c r="O41" s="1" t="n">
-        <v>46194</v>
+        <v>46265</v>
       </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 02:01)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RESERVA hora con Dentista</t>
+          <t>ASISTIR hora con Dentista (11:00 AM)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -1320,7 +1320,7 @@
         <v>46185</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>46194</v>
+        <v>46207</v>
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: Gantt pro + horas en tarjetas + cache SHA + limpieza REUNIONES
- Elimina hoja REUNIONES del Excel y todas sus referencias en código
- Agrega badge de ESFUERZO_HRS (ej. 1.5h) en tarjetas de Calendario,
  Kanban y Agenda del Día — solo visible cuando hrs > 0
- Cache basado en SHA de GitHub (reemplaza mtime local): consistencia
  cross-session y tras push remotos; TTL 60s con fallback a mtime
- Módulo Gantt profesional (ECharts custom series): barras por proyecto,
  color por Prioridad/Estado/Proyecto, marcador HOY, zoom temporal,
  tooltip rico, KPIs de contexto y leyenda dinámica
- Documentación de proyecto: CONTEXTO.md, MEMORIA.md, ROADMAP.md

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1,15 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="REUNIONES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,7 +522,6 @@
           <t>REVISIÓN plan de abastecimiento CL038</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -563,16 +561,12 @@
       <c r="L2" t="n">
         <v>1.5</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>46180</v>
       </c>
-      <c r="O2" s="1" t="n">
+      <c r="O2" s="2" t="n">
         <v>46192</v>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -583,7 +577,6 @@
           <t>SEGUIMIENTO correo clínica MEDs (carpeta rendición Isapre)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -628,17 +621,15 @@
           <t>Clínica MEDs</t>
         </is>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="2" t="n">
         <v>46179</v>
       </c>
-      <c r="O3" s="1" t="n">
+      <c r="O3" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P3" s="1" t="n">
+      <c r="P3" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -649,7 +640,6 @@
           <t>LLEVAR formulario seguro (boletas terapía)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -689,16 +679,12 @@
       <c r="L4" t="n">
         <v>0.5</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46189</v>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -709,7 +695,6 @@
           <t>SEGUIMIENTO IConstruye (reportabilidad gastado a la fecha)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -754,17 +739,15 @@
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="2" t="n">
         <v>46181</v>
       </c>
-      <c r="O5" s="1" t="n">
+      <c r="O5" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P5" s="1" t="n">
+      <c r="P5" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -775,7 +758,6 @@
           <t>APROBAR contratos</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -815,18 +797,15 @@
       <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O6" s="1" t="n">
+      <c r="O6" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P6" s="1" t="n">
+      <c r="P6" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -837,7 +816,6 @@
           <t>Aprobar regularización equipos robados</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -877,16 +855,12 @@
       <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O7" s="1" t="n">
+      <c r="O7" s="2" t="n">
         <v>46189</v>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -897,7 +871,6 @@
           <t>VISITAR a mi tío</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -937,16 +910,12 @@
       <c r="L8" t="n">
         <v>2</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O8" s="1" t="n">
+      <c r="O8" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -957,7 +926,6 @@
           <t>PASAR aspiradora</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -997,18 +965,15 @@
       <c r="L9" t="n">
         <v>0.5</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O9" s="1" t="n">
+      <c r="O9" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="P9" s="1" t="n">
+      <c r="P9" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1019,7 +984,6 @@
           <t>HACER baño 2</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1059,16 +1023,12 @@
       <c r="L10" t="n">
         <v>0.5</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O10" s="1" t="n">
+      <c r="O10" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1079,7 +1039,6 @@
           <t>ENVIAR correo presentación directorio (diferido)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1124,17 +1083,15 @@
           <t>Directorio</t>
         </is>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O11" s="1" t="n">
+      <c r="O11" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="P11" s="1" t="n">
+      <c r="P11" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1145,7 +1102,6 @@
           <t>SOLICITAR a GB respaldos de acta de sesión de Directorios</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -1190,15 +1146,12 @@
           <t>GB</t>
         </is>
       </c>
-      <c r="N12" s="1" t="n">
+      <c r="N12" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O12" s="1" t="n">
+      <c r="O12" s="2" t="n">
         <v>46191</v>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1209,7 +1162,6 @@
           <t>ACTUALIZAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1249,16 +1201,12 @@
       <c r="L13" t="n">
         <v>2</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O13" s="1" t="n">
+      <c r="O13" s="2" t="n">
         <v>46189</v>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1269,7 +1217,6 @@
           <t>RESERVA hora con Javi Franco</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1314,15 +1261,12 @@
           <t>Javi Franco</t>
         </is>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O14" s="1" t="n">
+      <c r="O14" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1333,7 +1277,6 @@
           <t>GESTIONAR firma MPD</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1378,15 +1321,12 @@
           <t>MPD</t>
         </is>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O15" s="1" t="n">
+      <c r="O15" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1397,7 +1337,6 @@
           <t>GESTIONAR firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1442,15 +1381,12 @@
           <t>Salfa</t>
         </is>
       </c>
-      <c r="N16" s="1" t="n">
+      <c r="N16" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O16" s="1" t="n">
+      <c r="O16" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1461,7 +1397,6 @@
           <t>ENVIAR comunicado por día de vacaciones</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1501,16 +1436,12 @@
       <c r="L17" t="n">
         <v>0.5</v>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" s="1" t="n">
+      <c r="N17" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O17" s="1" t="n">
+      <c r="O17" s="2" t="n">
         <v>46189</v>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1521,7 +1452,6 @@
           <t>PRESENTAR Dashboard Control de áridos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1561,18 +1491,15 @@
       <c r="L18" t="n">
         <v>2</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" s="1" t="n">
+      <c r="N18" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O18" s="1" t="n">
+      <c r="O18" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P18" s="1" t="n">
+      <c r="P18" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1583,7 +1510,6 @@
           <t>LAVAR ropa</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1623,18 +1549,15 @@
       <c r="L19" t="n">
         <v>0.5</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" s="1" t="n">
+      <c r="N19" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O19" s="1" t="n">
+      <c r="O19" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P19" s="1" t="n">
+      <c r="P19" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1645,7 +1568,6 @@
           <t>LAVAR losa</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1685,18 +1607,15 @@
       <c r="L20" t="n">
         <v>0.5</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" s="1" t="n">
+      <c r="N20" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O20" s="1" t="n">
+      <c r="O20" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P20" s="1" t="n">
+      <c r="P20" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1707,7 +1626,6 @@
           <t>CAPACITACIÓN Claude Code 3/5</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1747,16 +1665,12 @@
       <c r="L21" t="n">
         <v>2</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" s="1" t="n">
+      <c r="N21" s="2" t="n">
         <v>46181</v>
       </c>
-      <c r="O21" s="1" t="n">
+      <c r="O21" s="2" t="n">
         <v>46189</v>
       </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1767,7 +1681,6 @@
           <t>CAPACITACIÓN Claude Code 4/5</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1807,16 +1720,12 @@
       <c r="L22" t="n">
         <v>2</v>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" s="1" t="n">
+      <c r="N22" s="2" t="n">
         <v>46181</v>
       </c>
-      <c r="O22" s="1" t="n">
+      <c r="O22" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1827,7 +1736,6 @@
           <t>CAPACITACIÓN Claude Code 5/5</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1867,16 +1775,12 @@
       <c r="L23" t="n">
         <v>2</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" s="1" t="n">
+      <c r="N23" s="2" t="n">
         <v>46181</v>
       </c>
-      <c r="O23" s="1" t="n">
+      <c r="O23" s="2" t="n">
         <v>46191</v>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1887,7 +1791,6 @@
           <t>BARRER hojas</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1927,18 +1830,15 @@
       <c r="L24" t="n">
         <v>0.5</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" s="1" t="n">
+      <c r="N24" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O24" s="1" t="n">
+      <c r="O24" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P24" s="1" t="n">
+      <c r="P24" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1949,7 +1849,6 @@
           <t>PREPARAR almuerzo</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1989,18 +1888,15 @@
       <c r="L25" t="n">
         <v>0.5</v>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" s="1" t="n">
+      <c r="N25" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O25" s="1" t="n">
+      <c r="O25" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P25" s="1" t="n">
+      <c r="P25" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2011,7 +1907,6 @@
           <t>CAPACITACIÓN Claude Code 2/5</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2051,16 +1946,12 @@
       <c r="L26" t="n">
         <v>2</v>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" s="1" t="n">
+      <c r="N26" s="2" t="n">
         <v>46181</v>
       </c>
-      <c r="O26" s="1" t="n">
+      <c r="O26" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2071,7 +1962,6 @@
           <t>LLAMAR a Claudio S.</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2116,15 +2006,12 @@
           <t>Claudio S.</t>
         </is>
       </c>
-      <c r="N27" s="1" t="n">
+      <c r="N27" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O27" s="1" t="n">
+      <c r="O27" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2135,7 +2022,6 @@
           <t>ASISTIR cumpleaños Felipe M.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2175,18 +2061,15 @@
       <c r="L28" t="n">
         <v>2</v>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" s="1" t="n">
+      <c r="N28" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O28" s="1" t="n">
+      <c r="O28" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P28" s="1" t="n">
+      <c r="P28" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2197,7 +2080,6 @@
           <t>ASISTIR cumpleaños Esteban</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2237,18 +2119,15 @@
       <c r="L29" t="n">
         <v>2</v>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" s="1" t="n">
+      <c r="N29" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O29" s="1" t="n">
+      <c r="O29" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P29" s="1" t="n">
+      <c r="P29" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2259,7 +2138,6 @@
           <t>ENVIAR formato control de hormigones CL038</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -2299,16 +2177,12 @@
       <c r="L30" t="n">
         <v>0.5</v>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" s="1" t="n">
+      <c r="N30" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O30" s="1" t="n">
+      <c r="O30" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2319,7 +2193,6 @@
           <t>PRESENTAR carpetas 2 ciclos fertilización en isapre</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -2364,15 +2237,12 @@
           <t>Isapre</t>
         </is>
       </c>
-      <c r="N31" s="1" t="n">
+      <c r="N31" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O31" s="1" t="n">
+      <c r="O31" s="2" t="n">
         <v>46193</v>
       </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2383,7 +2253,6 @@
           <t>REVISIÓN funcionamiento KIT en IConstruye</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -2428,15 +2297,12 @@
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N32" s="1" t="n">
+      <c r="N32" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O32" s="1" t="n">
+      <c r="O32" s="2" t="n">
         <v>46191</v>
       </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2447,7 +2313,6 @@
           <t>ACTUALIZAR modelo Claude (validar datos)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2487,16 +2352,12 @@
       <c r="L33" t="n">
         <v>2</v>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" s="1" t="n">
+      <c r="N33" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O33" s="1" t="n">
+      <c r="O33" s="2" t="n">
         <v>46191</v>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2507,7 +2368,6 @@
           <t>COORDINAR hora psiquiatra (Consultar con la Lore)</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2552,17 +2412,15 @@
           <t>Consultorio</t>
         </is>
       </c>
-      <c r="N34" s="1" t="n">
+      <c r="N34" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O34" s="1" t="n">
+      <c r="O34" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="P34" s="1" t="n">
+      <c r="P34" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2573,7 +2431,6 @@
           <t>COMPRAR nuevo anillo matrimonial</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2613,16 +2470,12 @@
       <c r="L35" t="n">
         <v>1</v>
       </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" s="1" t="n">
+      <c r="N35" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O35" s="1" t="n">
+      <c r="O35" s="2" t="n">
         <v>46193</v>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2633,7 +2486,6 @@
           <t>ENVIAR a reparar bicicleta</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2673,16 +2525,12 @@
       <c r="L36" t="n">
         <v>0.5</v>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" s="1" t="n">
+      <c r="N36" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="O36" s="1" t="n">
+      <c r="O36" s="2" t="n">
         <v>46193</v>
       </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2693,7 +2541,6 @@
           <t>ENTRENAR trote: Rodaje 5K (Matutino)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2733,18 +2580,15 @@
       <c r="L37" t="n">
         <v>1</v>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" s="1" t="n">
+      <c r="N37" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O37" s="1" t="n">
+      <c r="O37" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P37" s="1" t="n">
+      <c r="P37" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2755,7 +2599,6 @@
           <t>ARMAR propuesta para salida fin de mes</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2795,16 +2638,12 @@
       <c r="L38" t="n">
         <v>1.5</v>
       </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" s="1" t="n">
+      <c r="N38" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="O38" s="1" t="n">
+      <c r="O38" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2815,7 +2654,6 @@
           <t>Revisar propuestas PUC RSC</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2855,14 +2693,9 @@
       <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" s="1" t="n">
+      <c r="N39" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2873,7 +2706,6 @@
           <t>Consolidar ensayos Mov. Tierra CL027</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2913,14 +2745,9 @@
       <c r="L40" t="n">
         <v>2</v>
       </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" s="1" t="n">
+      <c r="N40" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2931,7 +2758,6 @@
           <t>PEDIR hora psiquiatra</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2971,16 +2797,12 @@
       <c r="L41" t="n">
         <v>1</v>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" s="1" t="n">
+      <c r="N41" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="O41" s="1" t="n">
+      <c r="O41" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2991,7 +2813,6 @@
           <t>COMPRAR parafina</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3031,18 +2852,15 @@
       <c r="L42" t="n">
         <v>1</v>
       </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" s="1" t="n">
+      <c r="N42" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="O42" s="1" t="n">
+      <c r="O42" s="2" t="n">
         <v>46187</v>
       </c>
-      <c r="P42" s="1" t="n">
+      <c r="P42" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3053,7 +2871,6 @@
           <t>ENVIAR correo a Julián por empresa seguridad Moreno</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3093,18 +2910,15 @@
       <c r="L43" t="n">
         <v>1</v>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" s="1" t="n">
+      <c r="N43" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="O43" s="1" t="n">
+      <c r="O43" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P43" s="1" t="n">
+      <c r="P43" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3115,7 +2929,6 @@
           <t>REVISIÓN  con asesor de auto evaluación Sello PRO</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3155,16 +2968,12 @@
       <c r="L44" t="n">
         <v>1</v>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" s="1" t="n">
+      <c r="N44" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="O44" s="1" t="n">
+      <c r="O44" s="2" t="n">
         <v>46190</v>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3175,13 +2984,11 @@
           <t>ENVIAR pronostico polla mundialera 15-6-26</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -3202,19 +3009,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" s="1" t="n">
+      <c r="N45" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="O45" s="1" t="n">
+      <c r="O45" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3306,10 +3106,10 @@
           <t>Funcionamiento KIT y reporte reportabilidad</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -3352,10 +3152,10 @@
           <t>Respaldos actas de sesión Directorio</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>46183</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -3398,10 +3198,10 @@
           <t>Firma contrato pendiente</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -3444,10 +3244,10 @@
           <t>Firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -3490,10 +3290,10 @@
           <t>Presentación carpetas 2 ciclos fertilización</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>46179</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="G6" s="2" t="n">
         <v>46179</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -3536,10 +3336,10 @@
           <t>Correo rendición Isapre</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>46179</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="G7" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="H7" t="inlineStr">
@@ -3555,281 +3355,6 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>Correo recibido</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>TITULO</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>FECHA</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>TIPO</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>PARTICIPANTES</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ESTADO</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>COMPROMISO</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>RESPONSABLE_COMP</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>FECHA_COMP</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>ESTADO_COMP</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Reunión Directorio — Estado de Obras</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>46193</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Directorio</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Gerencia, Directores, ITO</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Preparar presentación estado obras; Enviar correo previo con agenda</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Juan</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>46191</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>En Proceso</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Presentar avance CL038 y CL027</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Coordinación Avance CL038</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>46190</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Obra</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ITO, Administrador de Obra, Subcontratistas</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Enviar informe de avance; Actualizar formato hormigones</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Juan</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>46189</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Revisar plan de abastecimiento áridos</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Revisión Contratos — Salfa / MPD</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>46189</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Contratos</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Gerencia, Asesor Legal, Representante Salfa</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Gestionar firma MPD; Gestionar firma Salfa; Enviar copia a legal</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Juan</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>En Proceso</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Confirmar asistencia de ambas partes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Seguimiento IConstruye — Funcionalidades</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>46191</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Tecnología</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Soporte IConstruye, Planificación</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Resolver funcionamiento KIT; Revisar reportabilidad gastado</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Juan</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>46191</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Preparar pantallazos con el error</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 13:42)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TAREAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TERCEROS" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,10 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,7 @@
           <t>REVISIÓN plan de abastecimiento CL038</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -561,12 +562,16 @@
       <c r="L2" t="n">
         <v>1.5</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="O2" s="1" t="n">
         <v>46198</v>
       </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -577,6 +582,7 @@
           <t>SEGUIMIENTO correo clínica MEDs (carpeta rendición Isapre)</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -621,15 +627,17 @@
           <t>Clínica MEDs</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="O3" s="2" t="n">
+      <c r="O3" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="1" t="n">
         <v>46186</v>
       </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -640,6 +648,7 @@
           <t>LLEVAR formulario seguro (boletas terapía)</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -679,12 +688,16 @@
       <c r="L4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -695,6 +708,7 @@
           <t>SEGUIMIENTO IConstruye (reportabilidad gastado a la fecha)</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -739,15 +753,17 @@
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="P5" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -758,6 +774,7 @@
           <t>APROBAR contratos</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -797,15 +814,18 @@
       <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O6" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="P6" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -816,6 +836,7 @@
           <t>Aprobar regularización equipos robados</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -855,15 +876,18 @@
       <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="1" t="n">
         <v>46191</v>
       </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -874,6 +898,7 @@
           <t>VISITAR a mi tío</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -913,12 +938,16 @@
       <c r="L8" t="n">
         <v>2</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="O8" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -929,6 +958,7 @@
           <t>PASAR aspiradora</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -968,15 +998,18 @@
       <c r="L9" t="n">
         <v>0.5</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O9" s="2" t="n">
+      <c r="O9" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -987,6 +1020,7 @@
           <t>HACER baño 2</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1026,12 +1060,16 @@
       <c r="L10" t="n">
         <v>0.5</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="O10" s="1" t="n">
         <v>46194</v>
       </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1042,6 +1080,7 @@
           <t>ENVIAR correo presentación directorio (diferido)</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1086,15 +1125,17 @@
           <t>Directorio</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="O11" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="P11" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1105,6 +1146,7 @@
           <t>SOLICITAR a GB respaldos de acta de sesión de Directorios</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -1149,12 +1191,15 @@
           <t>GB</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O12" s="2" t="n">
+      <c r="O12" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1165,6 +1210,7 @@
           <t>ACTUALIZAR formato control de hormigones CL038</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1204,12 +1250,16 @@
       <c r="L13" t="n">
         <v>1</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="O13" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1220,6 +1270,7 @@
           <t>ASISTIR hora con Dentista (11:00 AM)</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1264,12 +1315,15 @@
           <t>Javi Franco</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O14" s="2" t="n">
+      <c r="O14" s="1" t="n">
         <v>46207</v>
       </c>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1280,6 +1334,7 @@
           <t>GESTIONAR firma MPD</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1324,12 +1379,15 @@
           <t>MPD</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O15" s="2" t="n">
+      <c r="O15" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1340,6 +1398,7 @@
           <t>GESTIONAR firma Contrato Salfa-Londres</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1384,12 +1443,15 @@
           <t>Salfa</t>
         </is>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="N16" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="O16" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1400,6 +1462,7 @@
           <t>ENVIAR comunicado por día de vacaciones</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1439,15 +1502,18 @@
       <c r="L17" t="n">
         <v>0.5</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O17" s="2" t="n">
+      <c r="O17" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1458,6 +1524,7 @@
           <t>PRESENTAR Dashboard Control de áridos</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -1497,15 +1564,18 @@
       <c r="L18" t="n">
         <v>2</v>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O18" s="2" t="n">
+      <c r="O18" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1516,6 +1586,7 @@
           <t>LAVAR ropa</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1555,15 +1626,18 @@
       <c r="L19" t="n">
         <v>0.5</v>
       </c>
-      <c r="N19" s="2" t="n">
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O19" s="2" t="n">
+      <c r="O19" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P19" s="2" t="n">
+      <c r="P19" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1574,6 +1648,7 @@
           <t>LAVAR losa</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1613,15 +1688,18 @@
       <c r="L20" t="n">
         <v>0.5</v>
       </c>
-      <c r="N20" s="2" t="n">
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O20" s="2" t="n">
+      <c r="O20" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P20" s="2" t="n">
+      <c r="P20" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1632,6 +1710,7 @@
           <t>CAPACITACIÓN Claude Code 3/5</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1671,12 +1750,16 @@
       <c r="L21" t="n">
         <v>0.5</v>
       </c>
-      <c r="N21" s="2" t="n">
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O21" s="2" t="n">
+      <c r="O21" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1687,6 +1770,7 @@
           <t>CAPACITACIÓN Claude Code 4/5</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1726,12 +1810,16 @@
       <c r="L22" t="n">
         <v>0.5</v>
       </c>
-      <c r="N22" s="2" t="n">
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O22" s="2" t="n">
+      <c r="O22" s="1" t="n">
         <v>46197</v>
       </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1742,6 +1830,7 @@
           <t>CAPACITACIÓN Claude Code 5/5</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1781,12 +1870,16 @@
       <c r="L23" t="n">
         <v>0.5</v>
       </c>
-      <c r="N23" s="2" t="n">
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O23" s="2" t="n">
+      <c r="O23" s="1" t="n">
         <v>46198</v>
       </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1797,6 +1890,7 @@
           <t>BARRER hojas</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1836,15 +1930,18 @@
       <c r="L24" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="2" t="n">
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O24" s="2" t="n">
+      <c r="O24" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1855,6 +1952,7 @@
           <t>PREPARAR almuerzo</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1894,15 +1992,18 @@
       <c r="L25" t="n">
         <v>0.5</v>
       </c>
-      <c r="N25" s="2" t="n">
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O25" s="2" t="n">
+      <c r="O25" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1913,6 +2014,7 @@
           <t>CAPACITACIÓN Claude Code 2/5</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -1952,15 +2054,18 @@
       <c r="L26" t="n">
         <v>2</v>
       </c>
-      <c r="N26" s="2" t="n">
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="O26" s="2" t="n">
+      <c r="O26" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P26" s="2" t="n">
+      <c r="P26" s="1" t="n">
         <v>46189</v>
       </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1971,6 +2076,7 @@
           <t>LLAMAR a Claudio S.</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2015,12 +2121,15 @@
           <t>Claudio S.</t>
         </is>
       </c>
-      <c r="N27" s="2" t="n">
+      <c r="N27" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O27" s="2" t="n">
+      <c r="O27" s="1" t="n">
         <v>46199</v>
       </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2031,6 +2140,7 @@
           <t>ASISTIR cumpleaños Felipe M.</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2070,15 +2180,18 @@
       <c r="L28" t="n">
         <v>2</v>
       </c>
-      <c r="N28" s="2" t="n">
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O28" s="2" t="n">
+      <c r="O28" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2089,6 +2202,7 @@
           <t>ASISTIR cumpleaños Esteban</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2128,15 +2242,18 @@
       <c r="L29" t="n">
         <v>2</v>
       </c>
-      <c r="N29" s="2" t="n">
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O29" s="2" t="n">
+      <c r="O29" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P29" s="2" t="n">
+      <c r="P29" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2147,6 +2264,7 @@
           <t>ENVIAR formato control de hormigones CL038</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -2186,12 +2304,16 @@
       <c r="L30" t="n">
         <v>0.5</v>
       </c>
-      <c r="N30" s="2" t="n">
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O30" s="2" t="n">
+      <c r="O30" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2202,6 +2324,7 @@
           <t>PRESENTAR carpetas 2 ciclos fertilización en isapre</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -2246,12 +2369,15 @@
           <t>Isapre</t>
         </is>
       </c>
-      <c r="N31" s="2" t="n">
+      <c r="N31" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O31" s="2" t="n">
+      <c r="O31" s="1" t="n">
         <v>46214</v>
       </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2262,6 +2388,7 @@
           <t>REVISIÓN funcionamiento KIT en IConstruye</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -2306,12 +2433,15 @@
           <t>IConstruye</t>
         </is>
       </c>
-      <c r="N32" s="2" t="n">
+      <c r="N32" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="O32" s="2" t="n">
+      <c r="O32" s="1" t="n">
         <v>46203</v>
       </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2322,6 +2452,7 @@
           <t>ACTUALIZAR modelo Claude (validar datos)</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2361,12 +2492,16 @@
       <c r="L33" t="n">
         <v>2</v>
       </c>
-      <c r="N33" s="2" t="n">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O33" s="2" t="n">
+      <c r="O33" s="1" t="n">
         <v>46197</v>
       </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2377,6 +2512,7 @@
           <t>COORDINAR hora psiquiatra (Consultar con la Lore)</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2421,15 +2557,17 @@
           <t>Consultorio</t>
         </is>
       </c>
-      <c r="N34" s="2" t="n">
+      <c r="N34" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O34" s="2" t="n">
+      <c r="O34" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="P34" s="2" t="n">
+      <c r="P34" s="1" t="n">
         <v>46187</v>
       </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2440,6 +2578,7 @@
           <t>COMPRAR nuevo anillo matrimonial</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2479,12 +2618,16 @@
       <c r="L35" t="n">
         <v>1</v>
       </c>
-      <c r="N35" s="2" t="n">
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O35" s="2" t="n">
+      <c r="O35" s="1" t="n">
         <v>46214</v>
       </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2495,6 +2638,7 @@
           <t>ENVIAR a reparar bicicleta</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2534,12 +2678,16 @@
       <c r="L36" t="n">
         <v>0.5</v>
       </c>
-      <c r="N36" s="2" t="n">
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="O36" s="2" t="n">
+      <c r="O36" s="1" t="n">
         <v>46207</v>
       </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2550,6 +2698,7 @@
           <t>ENTRENAR trote: Rodaje 5K (Matutino)</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2589,15 +2738,18 @@
       <c r="L37" t="n">
         <v>1</v>
       </c>
-      <c r="N37" s="2" t="n">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O37" s="2" t="n">
+      <c r="O37" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P37" s="2" t="n">
+      <c r="P37" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2608,6 +2760,7 @@
           <t>ARMAR propuesta para salida fin de mes</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2647,15 +2800,18 @@
       <c r="L38" t="n">
         <v>1.5</v>
       </c>
-      <c r="N38" s="2" t="n">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="O38" s="2" t="n">
+      <c r="O38" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2666,6 +2822,7 @@
           <t>Revisar propuestas PUC RSC</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2705,9 +2862,14 @@
       <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="N39" s="2" t="n">
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" s="1" t="n">
         <v>46182</v>
       </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2718,6 +2880,7 @@
           <t>Consolidar ensayos Mov. Tierra CL027</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2757,9 +2920,14 @@
       <c r="L40" t="n">
         <v>2</v>
       </c>
-      <c r="N40" s="2" t="n">
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" s="1" t="n">
         <v>46182</v>
       </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2770,6 +2938,7 @@
           <t>ASISTIR hora psiquiatra (14 hrs. Lo Barnechea)</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2809,12 +2978,16 @@
       <c r="L41" t="n">
         <v>1</v>
       </c>
-      <c r="N41" s="2" t="n">
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="O41" s="2" t="n">
+      <c r="O41" s="1" t="n">
         <v>46265</v>
       </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2825,6 +2998,7 @@
           <t>COMPRAR parafina</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2864,15 +3038,18 @@
       <c r="L42" t="n">
         <v>1</v>
       </c>
-      <c r="N42" s="2" t="n">
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="O42" s="2" t="n">
+      <c r="O42" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="P42" s="2" t="n">
+      <c r="P42" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2883,6 +3060,7 @@
           <t>ENVIAR correo a Julián por empresa seguridad Moreno</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2922,15 +3100,18 @@
       <c r="L43" t="n">
         <v>1</v>
       </c>
-      <c r="N43" s="2" t="n">
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="O43" s="2" t="n">
+      <c r="O43" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P43" s="2" t="n">
+      <c r="P43" s="1" t="n">
         <v>46188</v>
       </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2941,6 +3122,7 @@
           <t>REVISIÓN  con asesor de auto evaluación Sello PRO</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -2980,15 +3162,18 @@
       <c r="L44" t="n">
         <v>1</v>
       </c>
-      <c r="N44" s="2" t="n">
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="O44" s="2" t="n">
+      <c r="O44" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="P44" s="2" t="n">
+      <c r="P44" s="1" t="n">
         <v>46191</v>
       </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2999,6 +3184,7 @@
           <t>ENVIAR pronostico polla mundialera 15-6-26</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -3038,15 +3224,18 @@
       <c r="L45" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="2" t="n">
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="O45" s="2" t="n">
+      <c r="O45" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="P45" s="2" t="n">
+      <c r="P45" s="1" t="n">
         <v>46189</v>
       </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3057,6 +3246,7 @@
           <t>CORRER 7K</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -3096,15 +3286,18 @@
       <c r="L46" t="n">
         <v>1</v>
       </c>
-      <c r="N46" s="2" t="n">
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="O46" s="2" t="n">
+      <c r="O46" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="P46" s="2" t="n">
+      <c r="P46" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3115,6 +3308,7 @@
           <t>ACTUALIZAR  Plan de Abastecimiento</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3154,12 +3348,16 @@
       <c r="L47" t="n">
         <v>0.5</v>
       </c>
-      <c r="N47" s="2" t="n">
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="O47" s="2" t="n">
+      <c r="O47" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3170,6 +3368,7 @@
           <t>APROBAR EEPP</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3209,12 +3408,16 @@
       <c r="L48" t="n">
         <v>2</v>
       </c>
-      <c r="N48" s="2" t="n">
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O48" s="2" t="n">
+      <c r="O48" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3225,6 +3428,7 @@
           <t>APROBAR OC</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3264,12 +3468,16 @@
       <c r="L49" t="n">
         <v>1.5</v>
       </c>
-      <c r="N49" s="2" t="n">
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O49" s="2" t="n">
+      <c r="O49" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3280,6 +3488,7 @@
           <t>APROBAR contratos</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3319,12 +3528,16 @@
       <c r="L50" t="n">
         <v>1.5</v>
       </c>
-      <c r="N50" s="2" t="n">
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O50" s="2" t="n">
+      <c r="O50" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3335,6 +3548,7 @@
           <t>VIAJAR a Olmue</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -3374,12 +3588,16 @@
       <c r="L51" t="n">
         <v>1</v>
       </c>
-      <c r="N51" s="2" t="n">
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O51" s="2" t="n">
+      <c r="O51" s="1" t="n">
         <v>46198</v>
       </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3390,6 +3608,7 @@
           <t>LAVAR ropa</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3429,12 +3648,16 @@
       <c r="L52" t="n">
         <v>1</v>
       </c>
-      <c r="N52" s="2" t="n">
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O52" s="2" t="n">
+      <c r="O52" s="1" t="n">
         <v>46196</v>
       </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3445,6 +3668,7 @@
           <t>ENTRENAMIENTO fuerza</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>Tarea</t>
@@ -3484,12 +3708,16 @@
       <c r="L53" t="n">
         <v>1</v>
       </c>
-      <c r="N53" s="2" t="n">
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O53" s="2" t="n">
+      <c r="O53" s="1" t="n">
         <v>46195</v>
       </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3500,6 +3728,7 @@
           <t>VISITAR escuela construcción PUC</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Compromiso</t>
@@ -3539,12 +3768,70 @@
       <c r="L54" t="n">
         <v>1</v>
       </c>
-      <c r="N54" s="2" t="n">
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="O54" s="2" t="n">
+      <c r="O54" s="1" t="n">
         <v>46197</v>
       </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ACTUALIZACIÓN plano AV (Helsby)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>CL027</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O55" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3636,10 +3923,10 @@
           <t>Funcionamiento KIT y reporte reportabilidad</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -3682,10 +3969,10 @@
           <t>Respaldos actas de sesión Directorio</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -3728,10 +4015,10 @@
           <t>Firma contrato pendiente</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -3774,10 +4061,10 @@
           <t>Firma Contrato Salfa-Londres</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -3820,10 +4107,10 @@
           <t>Presentación carpetas 2 ciclos fertilización</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>46179</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -3866,10 +4153,10 @@
           <t>Correo rendición Isapre</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>46186</v>
       </c>
       <c r="H7" t="inlineStr">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 13:45)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3780,6 +3780,56 @@
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ACTIVAR rol reportes a Jefes de Proyectos AT</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="O55" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 13:47)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3796,7 +3796,11 @@
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>Trabajo</t>
@@ -3817,9 +3821,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="J55" t="n">
+        <v>3</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.5</v>
+      </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" s="1" t="n">
         <v>46195</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 14:19)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1362,7 +1362,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Esperando Terceros</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1385,7 +1385,9 @@
       <c r="O15" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 14:38)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -760,7 +760,7 @@
         <v>46195</v>
       </c>
       <c r="P5" s="1" t="n">
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 15:12)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3822,7 +3822,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -3841,7 +3841,9 @@
       <c r="O55" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="P55" t="inlineStr"/>
+      <c r="P55" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (22/06 19:22)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1058,14 +1058,14 @@
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 13:53)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -693,7 +693,7 @@
         <v>46183</v>
       </c>
       <c r="O4" s="1" t="n">
-        <v>46196</v>
+        <v>46203</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
         <v>46183</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>46203</v>
+        <v>46196</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 13:54)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -693,7 +693,7 @@
         <v>46183</v>
       </c>
       <c r="O4" s="1" t="n">
-        <v>46203</v>
+        <v>46196</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
@@ -1759,7 +1759,7 @@
         <v>46181</v>
       </c>
       <c r="O21" s="1" t="n">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 13:55)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -693,7 +693,7 @@
         <v>46183</v>
       </c>
       <c r="O4" s="1" t="n">
-        <v>46203</v>
+        <v>46196</v>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
         <v>46183</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>46196</v>
+        <v>46203</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 13:56)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1195,7 +1195,7 @@
         <v>46183</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>46199</v>
+        <v>46196</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
@@ -1759,7 +1759,7 @@
         <v>46181</v>
       </c>
       <c r="O21" s="1" t="n">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:21)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1017,7 +1017,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HACER baño 2</t>
+          <t>HACER baño 2 (tina)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1065,7 +1065,7 @@
         <v>46185</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:26)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3846,6 +3846,56 @@
       </c>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ENVIAR contrato AUTER a Eduardo Fuentes</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O56" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:29)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,11 @@
           <t>COMENTARIOS</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ORDEN</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -572,6 +577,9 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -638,6 +646,9 @@
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -698,6 +709,9 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -764,6 +778,9 @@
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -826,6 +843,9 @@
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -888,6 +908,9 @@
       </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -948,6 +971,9 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1010,6 +1036,9 @@
       </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1070,6 +1099,9 @@
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1136,6 +1168,9 @@
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1200,6 +1235,9 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1260,6 +1298,9 @@
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
+      <c r="S13" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1324,6 +1365,9 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1390,6 +1434,9 @@
       </c>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1456,6 +1503,9 @@
       </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
+      <c r="S16" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1518,6 +1568,9 @@
       </c>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1580,6 +1633,9 @@
       </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
+      <c r="S18" t="n">
+        <v>160</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1642,6 +1698,9 @@
       </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
+      <c r="S19" t="n">
+        <v>170</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1704,6 +1763,9 @@
       </c>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
+      <c r="S20" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1764,6 +1826,9 @@
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
+      <c r="S21" t="n">
+        <v>190</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1824,6 +1889,9 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
+      <c r="S22" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1884,6 +1952,9 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
+      <c r="S23" t="n">
+        <v>210</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1946,6 +2017,9 @@
       </c>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
+      <c r="S24" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2008,6 +2082,9 @@
       </c>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
+      <c r="S25" t="n">
+        <v>230</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2070,6 +2147,9 @@
       </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
+      <c r="S26" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2134,6 +2214,9 @@
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
+      <c r="S27" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2196,6 +2279,9 @@
       </c>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
+      <c r="S28" t="n">
+        <v>260</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2258,6 +2344,9 @@
       </c>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
+      <c r="S29" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2318,6 +2407,9 @@
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2382,6 +2474,9 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
+      <c r="S31" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2446,6 +2541,9 @@
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
+      <c r="S32" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2506,6 +2604,9 @@
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
+      <c r="S33" t="n">
+        <v>310</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2572,6 +2673,9 @@
       </c>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
+      <c r="S34" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2632,6 +2736,9 @@
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
+      <c r="S35" t="n">
+        <v>330</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2692,6 +2799,9 @@
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
+      <c r="S36" t="n">
+        <v>340</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2754,6 +2864,9 @@
       </c>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
+      <c r="S37" t="n">
+        <v>350</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2816,6 +2929,9 @@
       </c>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
+      <c r="S38" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2874,6 +2990,9 @@
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
+      <c r="S39" t="n">
+        <v>370</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2932,6 +3051,9 @@
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
+      <c r="S40" t="n">
+        <v>380</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2992,6 +3114,9 @@
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
+      <c r="S41" t="n">
+        <v>390</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3054,6 +3179,9 @@
       </c>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
+      <c r="S42" t="n">
+        <v>400</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3116,6 +3244,9 @@
       </c>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
+      <c r="S43" t="n">
+        <v>410</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3178,6 +3309,9 @@
       </c>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
+      <c r="S44" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3240,6 +3374,9 @@
       </c>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
+      <c r="S45" t="n">
+        <v>430</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3302,6 +3439,9 @@
       </c>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
+      <c r="S46" t="n">
+        <v>440</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3362,6 +3502,9 @@
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
+      <c r="S47" t="n">
+        <v>450</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3422,6 +3565,9 @@
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
+      <c r="S48" t="n">
+        <v>460</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3482,6 +3628,9 @@
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
+      <c r="S49" t="n">
+        <v>470</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3542,6 +3691,9 @@
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
+      <c r="S50" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3602,6 +3754,9 @@
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
+      <c r="S51" t="n">
+        <v>490</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3662,6 +3817,9 @@
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr"/>
+      <c r="S52" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3724,6 +3882,9 @@
       </c>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
+      <c r="S53" t="n">
+        <v>510</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3784,6 +3945,9 @@
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
+      <c r="S54" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3846,6 +4010,9 @@
       </c>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
+      <c r="S55" t="n">
+        <v>530</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3862,7 +4029,11 @@
           <t>Tarea</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>Trabajo</t>
@@ -3883,9 +4054,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="J56" t="n">
+        <v>3</v>
+      </c>
+      <c r="K56" t="n">
+        <v>3</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1</v>
+      </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="1" t="n">
         <v>46196</v>
@@ -3896,6 +4073,60 @@
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
+      <c r="S56" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ASISTIR cumpleaños prima</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O57" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:43)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3933,7 +3933,7 @@
         <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" s="1" t="n">
@@ -4092,7 +4092,11 @@
           <t>Compromiso</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>Personal</t>
@@ -4113,9 +4117,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="J57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" t="n">
+        <v>3</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1</v>
+      </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" s="1" t="n">
         <v>46196</v>
@@ -4126,7 +4136,9 @@
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="S57" t="n">
+        <v>550</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:56)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1100,7 +1100,7 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>80</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11">
@@ -1299,7 +1299,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>110</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -2408,7 +2408,7 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>280</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31">
@@ -3503,7 +3503,7 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>450</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48">
@@ -3566,7 +3566,7 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="n">
-        <v>460</v>
+        <v>450</v>
       </c>
     </row>
     <row r="49">
@@ -3629,7 +3629,7 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
     </row>
     <row r="50">
@@ -3692,7 +3692,7 @@
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="51">
@@ -4139,7 +4139,7 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="n">
-        <v>550</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 14:57)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1299,7 +1299,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>280</v>
+        <v>450</v>
       </c>
     </row>
     <row r="14">
@@ -2408,7 +2408,7 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>450</v>
+        <v>460</v>
       </c>
     </row>
     <row r="31">
@@ -3503,7 +3503,7 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="48">
@@ -3629,7 +3629,7 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="n">
-        <v>470</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 15:14)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4141,6 +4141,61 @@
       <c r="S57" t="n">
         <v>480</v>
       </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>APROBAR EEPP (2/3)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Of. Central</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Gestión Corporativa</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="O58" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 15:15)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3638,7 +3638,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>APROBAR contratos</t>
+          <t>APROBAR contratos (1/3)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -4245,9 +4245,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="J59" t="n">
+        <v>3</v>
+      </c>
+      <c r="K59" t="n">
+        <v>3</v>
+      </c>
+      <c r="L59" t="n">
+        <v>1</v>
+      </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" s="1" t="n">
         <v>46196</v>
@@ -4258,7 +4264,9 @@
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
+      <c r="S59" t="n">
+        <v>570</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 15:16)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2592,7 +2592,7 @@
         <v>5</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" s="1" t="n">
@@ -4308,9 +4308,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="J60" t="n">
+        <v>3</v>
+      </c>
+      <c r="K60" t="n">
+        <v>3</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1</v>
+      </c>
       <c r="M60" t="inlineStr"/>
       <c r="N60" s="1" t="n">
         <v>46196</v>
@@ -4321,7 +4327,9 @@
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+      <c r="S60" t="n">
+        <v>580</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 17:04)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3543,7 +3543,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -3562,7 +3562,9 @@
       <c r="O48" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="P48" t="inlineStr"/>
+      <c r="P48" s="1" t="n">
+        <v>46196</v>
+      </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 20:05)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,6 +517,11 @@
           <t>ORDEN</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>HORAS_REALES</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -580,6 +585,9 @@
       <c r="S2" t="n">
         <v>0</v>
       </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -648,6 +656,9 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
         <v>10</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -712,6 +723,9 @@
       <c r="S4" t="n">
         <v>20</v>
       </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -781,6 +795,9 @@
       <c r="S5" t="n">
         <v>30</v>
       </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -846,6 +863,9 @@
       <c r="S6" t="n">
         <v>40</v>
       </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -910,6 +930,9 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
         <v>50</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -974,6 +997,9 @@
       <c r="S8" t="n">
         <v>60</v>
       </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1038,6 +1064,9 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
         <v>70</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1102,6 +1131,9 @@
       <c r="S10" t="n">
         <v>550</v>
       </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1170,6 +1202,9 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
         <v>90</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1238,6 +1273,9 @@
       <c r="S12" t="n">
         <v>100</v>
       </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1301,6 +1339,9 @@
       <c r="S13" t="n">
         <v>450</v>
       </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1368,6 +1409,9 @@
       <c r="S14" t="n">
         <v>120</v>
       </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1437,6 +1481,9 @@
       <c r="S15" t="n">
         <v>130</v>
       </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1506,6 +1553,9 @@
       <c r="S16" t="n">
         <v>140</v>
       </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1571,6 +1621,9 @@
       <c r="S17" t="n">
         <v>150</v>
       </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1636,6 +1689,9 @@
       <c r="S18" t="n">
         <v>160</v>
       </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1701,6 +1757,9 @@
       <c r="S19" t="n">
         <v>170</v>
       </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1765,6 +1824,9 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="n">
         <v>180</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1829,6 +1891,9 @@
       <c r="S21" t="n">
         <v>190</v>
       </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1892,6 +1957,9 @@
       <c r="S22" t="n">
         <v>200</v>
       </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1955,6 +2023,9 @@
       <c r="S23" t="n">
         <v>210</v>
       </c>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2020,6 +2091,9 @@
       <c r="S24" t="n">
         <v>220</v>
       </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2085,6 +2159,9 @@
       <c r="S25" t="n">
         <v>230</v>
       </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2149,6 +2226,9 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="n">
         <v>240</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -2217,6 +2297,9 @@
       <c r="S27" t="n">
         <v>250</v>
       </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2282,6 +2365,9 @@
       <c r="S28" t="n">
         <v>260</v>
       </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2346,6 +2432,9 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="n">
         <v>270</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2410,6 +2499,9 @@
       <c r="S30" t="n">
         <v>460</v>
       </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2477,6 +2569,9 @@
       <c r="S31" t="n">
         <v>290</v>
       </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2544,6 +2639,9 @@
       <c r="S32" t="n">
         <v>300</v>
       </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2607,6 +2705,9 @@
       <c r="S33" t="n">
         <v>310</v>
       </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2675,6 +2776,9 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
         <v>320</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2739,6 +2843,9 @@
       <c r="S35" t="n">
         <v>330</v>
       </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2802,6 +2909,9 @@
       <c r="S36" t="n">
         <v>340</v>
       </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2867,6 +2977,9 @@
       <c r="S37" t="n">
         <v>350</v>
       </c>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2931,6 +3044,9 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
         <v>360</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2993,6 +3109,9 @@
       <c r="S39" t="n">
         <v>370</v>
       </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3054,6 +3173,9 @@
       <c r="S40" t="n">
         <v>380</v>
       </c>
+      <c r="T40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3117,6 +3239,9 @@
       <c r="S41" t="n">
         <v>390</v>
       </c>
+      <c r="T41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3182,6 +3307,9 @@
       <c r="S42" t="n">
         <v>400</v>
       </c>
+      <c r="T42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3247,6 +3375,9 @@
       <c r="S43" t="n">
         <v>410</v>
       </c>
+      <c r="T43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3312,6 +3443,9 @@
       <c r="S44" t="n">
         <v>420</v>
       </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3377,6 +3511,9 @@
       <c r="S45" t="n">
         <v>430</v>
       </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3441,6 +3578,9 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="n">
         <v>440</v>
+      </c>
+      <c r="T46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3505,6 +3645,9 @@
       <c r="S47" t="n">
         <v>470</v>
       </c>
+      <c r="T47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3569,6 +3712,9 @@
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="n">
         <v>80</v>
+      </c>
+      <c r="T48" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3633,6 +3779,9 @@
       <c r="S49" t="n">
         <v>280</v>
       </c>
+      <c r="T49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3696,6 +3845,9 @@
       <c r="S50" t="n">
         <v>110</v>
       </c>
+      <c r="T50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3759,6 +3911,9 @@
       <c r="S51" t="n">
         <v>490</v>
       </c>
+      <c r="T51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3822,6 +3977,9 @@
       <c r="S52" t="n">
         <v>500</v>
       </c>
+      <c r="T52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3886,6 +4044,9 @@
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="n">
         <v>510</v>
+      </c>
+      <c r="T53" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -3950,6 +4111,9 @@
       <c r="S54" t="n">
         <v>520</v>
       </c>
+      <c r="T54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4015,6 +4179,9 @@
       <c r="S55" t="n">
         <v>530</v>
       </c>
+      <c r="T55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4079,6 +4246,9 @@
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="n">
         <v>540</v>
+      </c>
+      <c r="T56" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -4143,6 +4313,9 @@
       <c r="S57" t="n">
         <v>480</v>
       </c>
+      <c r="T57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4206,6 +4379,9 @@
       <c r="S58" t="n">
         <v>560</v>
       </c>
+      <c r="T58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4269,6 +4445,9 @@
       <c r="S59" t="n">
         <v>570</v>
       </c>
+      <c r="T59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4331,6 +4510,9 @@
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="n">
         <v>580</v>
+      </c>
+      <c r="T60" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4456,7 +4638,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gerencia Buenos Aires</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4502,7 +4684,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mandante Proyecto</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 21:06)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1129,7 +1129,7 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>550</v>
+        <v>110</v>
       </c>
       <c r="T10" t="n">
         <v>0</v>
@@ -1337,7 +1337,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -2295,7 +2295,7 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="T27" t="n">
         <v>0</v>
@@ -2497,7 +2497,7 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>460</v>
+        <v>290</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="T31" t="n">
         <v>0</v>
@@ -2703,7 +2703,7 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="n">
-        <v>310</v>
+        <v>450</v>
       </c>
       <c r="T33" t="n">
         <v>0</v>
@@ -3643,7 +3643,7 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="T47" t="n">
         <v>0</v>
@@ -3777,7 +3777,7 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="n">
-        <v>280</v>
+        <v>470</v>
       </c>
       <c r="T49" t="n">
         <v>0</v>
@@ -3843,7 +3843,7 @@
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="n">
-        <v>110</v>
+        <v>480</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
@@ -4311,7 +4311,7 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="n">
-        <v>480</v>
+        <v>550</v>
       </c>
       <c r="T57" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (23/06 22:53)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3754,7 +3754,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -3773,7 +3773,9 @@
       <c r="O49" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="P49" t="inlineStr"/>
+      <c r="P49" s="1" t="n">
+        <v>46196</v>
+      </c>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:44)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3890,7 +3890,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3909,7 +3909,9 @@
       <c r="O51" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="P51" t="inlineStr"/>
+      <c r="P51" s="1" t="n">
+        <v>46201</v>
+      </c>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:45)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -4426,7 +4426,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J59" t="n">
@@ -4445,7 +4445,9 @@
       <c r="O59" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="P59" t="inlineStr"/>
+      <c r="P59" s="1" t="n">
+        <v>46201</v>
+      </c>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:46)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -570,18 +570,22 @@
         <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" s="1" t="n">
         <v>46180</v>
       </c>
       <c r="O2" s="1" t="n">
-        <v>46198</v>
+        <v>46206</v>
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>[28/06/2026 14:46 🔄] FECHA_COMPROMISO: '25/06/2026' → '03/07/2026' | ESFUERZO_HRS: '1.5' → '1.0'</t>
+        </is>
+      </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:47)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -4308,7 +4308,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J57" t="n">
@@ -4327,7 +4327,9 @@
       <c r="O57" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="P57" t="inlineStr"/>
+      <c r="P57" s="1" t="n">
+        <v>46201</v>
+      </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:51)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2301,11 +2301,15 @@
         <v>46185</v>
       </c>
       <c r="O27" s="1" t="n">
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>[28/06/2026 14:51 🔄] FECHA_COMPROMISO: '26/06/2026' → '28/06/2026'</t>
+        </is>
+      </c>
       <c r="S27" t="n">
         <v>280</v>
       </c>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:52)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T60"/>
+  <dimension ref="A1:T59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4075,17 +4075,17 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VISITAR escuela construcción PUC</t>
+          <t>ACTIVAR rol reportes a Jefes de Proyectos AT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Compromiso</t>
+          <t>Tarea</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -4105,12 +4105,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completada</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -4120,20 +4120,22 @@
         <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" s="1" t="n">
         <v>46195</v>
       </c>
       <c r="O54" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="P54" t="inlineStr"/>
+        <v>46195</v>
+      </c>
+      <c r="P54" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="n">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="T54" t="n">
         <v>0</v>
@@ -4141,11 +4143,11 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ACTIVAR rol reportes a Jefes de Proyectos AT</t>
+          <t>ENVIAR contrato AUTER a Eduardo Fuentes</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -4186,22 +4188,22 @@
         <v>3</v>
       </c>
       <c r="L55" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" s="1" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="O55" s="1" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="P55" s="1" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="T55" t="n">
         <v>0</v>
@@ -4209,17 +4211,17 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ENVIAR contrato AUTER a Eduardo Fuentes</t>
+          <t>ASISTIR cumpleaños prima</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Tarea</t>
+          <t>Compromiso</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4229,12 +4231,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Trabajo</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Gestión Corporativa</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4254,7 +4256,7 @@
         <v>3</v>
       </c>
       <c r="L56" t="n">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="1" t="n">
@@ -4264,12 +4266,12 @@
         <v>46196</v>
       </c>
       <c r="P56" s="1" t="n">
-        <v>46196</v>
+        <v>46201</v>
       </c>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="T56" t="n">
         <v>0</v>
@@ -4277,37 +4279,37 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ASISTIR cumpleaños prima</t>
+          <t>APROBAR EEPP (2/3)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Compromiso</t>
+          <t>Tarea</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>Of. Central</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Trabajo</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Gestión Corporativa</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4322,14 +4324,14 @@
         <v>3</v>
       </c>
       <c r="L57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="O57" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="P57" s="1" t="n">
         <v>46201</v>
@@ -4337,7 +4339,7 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="T57" t="n">
         <v>0</v>
@@ -4345,11 +4347,11 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>APROBAR EEPP (2/3)</t>
+          <t>APROBAR contratos (2/3)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -4405,7 +4407,7 @@
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="T58" t="n">
         <v>0</v>
@@ -4413,11 +4415,11 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>APROBAR contratos (2/3)</t>
+          <t>APROBAR OC (2/3)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -4428,7 +4430,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Of. Central</t>
+          <t>CL038</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4473,77 +4475,9 @@
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="n">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="T59" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>APROBAR OC (2/3)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>CL038</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Trabajo</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Gestión Corporativa</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Completada</t>
-        </is>
-      </c>
-      <c r="J60" t="n">
-        <v>3</v>
-      </c>
-      <c r="K60" t="n">
-        <v>3</v>
-      </c>
-      <c r="L60" t="n">
-        <v>1</v>
-      </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" s="1" t="n">
-        <v>46196</v>
-      </c>
-      <c r="O60" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="P60" s="1" t="n">
-        <v>46201</v>
-      </c>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="n">
-        <v>580</v>
-      </c>
-      <c r="T60" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:53)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2035,11 +2035,15 @@
         <v>46181</v>
       </c>
       <c r="O23" s="1" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>[28/06/2026 14:53 🔄] FECHA_COMPROMISO: '27/06/2026' → '30/06/2026'</t>
+        </is>
+      </c>
       <c r="S23" t="n">
         <v>210</v>
       </c>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (28/06 14:54)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2729,11 +2729,15 @@
         <v>46183</v>
       </c>
       <c r="O33" s="1" t="n">
-        <v>46197</v>
+        <v>46202</v>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>[28/06/2026 14:54 🔄] FECHA_COMPROMISO: '24/06/2026' → '29/06/2026'</t>
+        </is>
+      </c>
       <c r="S33" t="n">
         <v>450</v>
       </c>

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (30/06 02:28)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -3673,13 +3673,14 @@
         <v>46190</v>
       </c>
       <c r="O47" s="1" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>[28/06/2026 14:53 🔄] FECHA_COMPROMISO: '23/06/2026' → '28/06/2026'</t>
+          <t>[30/06/2026 02:28 🔄] FECHA_COMPROMISO: '28/06/2026' → '30/06/2026'
+[28/06/2026 14:53 🔄] FECHA_COMPROMISO: '23/06/2026' → '28/06/2026'</t>
         </is>
       </c>
       <c r="S47" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (30/06 02:29)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1127,13 +1127,14 @@
         <v>46185</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>[28/06/2026 14:46 🔄] FECHA_COMPROMISO: '23/06/2026' → '29/06/2026'</t>
+          <t>[30/06/2026 02:29 🔄] FECHA_COMPROMISO: '29/06/2026' → '30/06/2026'
+[28/06/2026 14:46 🔄] FECHA_COMPROMISO: '23/06/2026' → '29/06/2026'</t>
         </is>
       </c>
       <c r="S10" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (30/06 02:30)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2314,13 +2314,14 @@
         <v>46185</v>
       </c>
       <c r="O27" s="1" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>[28/06/2026 14:51 🔄] FECHA_COMPROMISO: '26/06/2026' → '28/06/2026'</t>
+          <t>[30/06/2026 02:30 🔄] FECHA_COMPROMISO: '28/06/2026' → '30/06/2026'
+[28/06/2026 14:51 🔄] FECHA_COMPROMISO: '26/06/2026' → '28/06/2026'</t>
         </is>
       </c>
       <c r="S27" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (30/06 02:31)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -1896,13 +1896,14 @@
         <v>46181</v>
       </c>
       <c r="O21" s="1" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>[28/06/2026 14:52 🔄] FECHA_COMPROMISO: '26/06/2026' → '28/06/2026'</t>
+          <t>[30/06/2026 02:31 🔄] FECHA_COMPROMISO: '28/06/2026' → '30/06/2026'
+[28/06/2026 14:52 🔄] FECHA_COMPROMISO: '26/06/2026' → '28/06/2026'</t>
         </is>
       </c>
       <c r="S21" t="n">

</xml_diff>

<commit_message>
update: tareas actualizadas desde app (30/06 02:33)
</commit_message>
<xml_diff>
--- a/TAREAS_JOCHOA.xlsx
+++ b/TAREAS_JOCHOA.xlsx
@@ -2733,13 +2733,14 @@
         <v>46183</v>
       </c>
       <c r="O33" s="1" t="n">
-        <v>46202</v>
+        <v>46205</v>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>[28/06/2026 14:54 🔄] FECHA_COMPROMISO: '24/06/2026' → '29/06/2026'</t>
+          <t>[30/06/2026 02:33 🔄] FECHA_COMPROMISO: '29/06/2026' → '02/07/2026'
+[28/06/2026 14:54 🔄] FECHA_COMPROMISO: '24/06/2026' → '29/06/2026'</t>
         </is>
       </c>
       <c r="S33" t="n">

</xml_diff>